<commit_message>
Full text screening done
</commit_message>
<xml_diff>
--- a/04_fulltext_screening/fullTextScreening.xlsx
+++ b/04_fulltext_screening/fullTextScreening.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arjen/kDrive/Obsidian/Literature Review MDIM/04_fulltext_screening/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53884FC7-D03F-1443-812C-10031BEAD002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F603906-EEBF-ED44-8B9F-13DF7DBBF01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_CoreScreening" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="356">
   <si>
     <t>Auteur(s) en Jaar</t>
   </si>
@@ -1032,6 +1032,81 @@
   </si>
   <si>
     <t>Luca e.a. (2023)</t>
+  </si>
+  <si>
+    <t>Combining and presenting data on the city of Florence</t>
+  </si>
+  <si>
+    <t>On the Terragov project</t>
+  </si>
+  <si>
+    <t>Fuzzy ontology creation from unstructures data</t>
+  </si>
+  <si>
+    <t>No paper present</t>
+  </si>
+  <si>
+    <t>On ontology building</t>
+  </si>
+  <si>
+    <t>Brandenburg builds a ontlogy accoring to the EU rules</t>
+  </si>
+  <si>
+    <t>Thesis on using gegraphical ontologies for cultrual heratige</t>
+  </si>
+  <si>
+    <t>Using, legacy, Workflow, Service, life-event ontlogies to create a e-gov ontology</t>
+  </si>
+  <si>
+    <t>Non English</t>
+  </si>
+  <si>
+    <t>About integration of large datasets and performance</t>
+  </si>
+  <si>
+    <t>REMO for smart Energy Management</t>
+  </si>
+  <si>
+    <t>Building a huge mineral database and ontlogy</t>
+  </si>
+  <si>
+    <t>Building a data twin in India</t>
+  </si>
+  <si>
+    <t>EU Report on using AI for interoperability</t>
+  </si>
+  <si>
+    <t>Description of collaboration in Italy</t>
+  </si>
+  <si>
+    <t>Introduces loosly couplesd information world</t>
+  </si>
+  <si>
+    <t>Building a military system with a semantic layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discussion of th eupper ontlogy </t>
+  </si>
+  <si>
+    <t>Using Geo ontlogies in Bangladesh</t>
+  </si>
+  <si>
+    <t>Dissertatie over het verrijken van geodata om het semantisch te kunnen linken</t>
+  </si>
+  <si>
+    <t>Good foundation for semantic challenges and solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aligning semantics in healthcare </t>
+  </si>
+  <si>
+    <t>Building a ontology to detect fraud</t>
+  </si>
+  <si>
+    <t>Dissertation on ontology alignment</t>
+  </si>
+  <si>
+    <t>No Full paper present</t>
   </si>
 </sst>
 </file>
@@ -5496,329 +5571,686 @@
     </row>
     <row r="2" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="25" t="s">
-        <v>329</v>
+        <v>302</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>328</v>
+        <v>303</v>
+      </c>
+      <c r="D2" s="23">
+        <v>2</v>
+      </c>
+      <c r="E2" s="23">
+        <v>2</v>
+      </c>
+      <c r="F2" s="23">
+        <v>1</v>
+      </c>
+      <c r="G2" s="23">
+        <v>1</v>
       </c>
       <c r="H2" s="24">
-        <f t="shared" ref="H2:H27" si="0">SUM(D2:G2)</f>
-        <v>0</v>
+        <f>SUM(D2:G2)</f>
+        <v>6</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>331</v>
+      </c>
+      <c r="K2" s="23" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="26" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>303</v>
+        <v>291</v>
+      </c>
+      <c r="D3" s="23">
+        <v>2</v>
+      </c>
+      <c r="E3" s="23">
+        <v>1</v>
+      </c>
+      <c r="F3" s="23">
+        <v>1</v>
+      </c>
+      <c r="G3" s="23">
+        <v>2</v>
       </c>
       <c r="H3" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D3:G3)</f>
+        <v>6</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="26" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>291</v>
+        <v>293</v>
+      </c>
+      <c r="D4" s="23">
+        <v>2</v>
+      </c>
+      <c r="E4" s="23">
+        <v>1</v>
+      </c>
+      <c r="F4" s="23">
+        <v>1</v>
+      </c>
+      <c r="G4" s="23">
+        <v>1</v>
       </c>
       <c r="H4" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D4:G4)</f>
+        <v>5</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="26" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>293</v>
+        <v>309</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>334</v>
       </c>
       <c r="H5" s="24">
-        <f t="shared" si="0"/>
+        <f>SUM(D5:G5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="26" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>309</v>
+        <v>295</v>
+      </c>
+      <c r="D6" s="23">
+        <v>0</v>
+      </c>
+      <c r="E6" s="23">
+        <v>1</v>
+      </c>
+      <c r="F6" s="23">
+        <v>1</v>
+      </c>
+      <c r="G6" s="23">
+        <v>2</v>
       </c>
       <c r="H6" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D6:G6)</f>
+        <v>4</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="26" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>295</v>
+        <v>307</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>334</v>
       </c>
       <c r="H7" s="24">
-        <f t="shared" si="0"/>
+        <f>SUM(D7:G7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="26" t="s">
-        <v>306</v>
+        <v>281</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>307</v>
+        <v>282</v>
+      </c>
+      <c r="D8" s="23">
+        <v>2</v>
+      </c>
+      <c r="E8" s="23">
+        <v>1</v>
+      </c>
+      <c r="F8" s="23">
+        <v>1</v>
+      </c>
+      <c r="G8" s="23">
+        <v>1</v>
       </c>
       <c r="H8" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D8:G8)</f>
+        <v>5</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="26" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>282</v>
+        <v>280</v>
+      </c>
+      <c r="D9" s="23">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23">
+        <v>2</v>
+      </c>
+      <c r="F9" s="23">
+        <v>1</v>
+      </c>
+      <c r="G9" s="23">
+        <v>2</v>
       </c>
       <c r="H9" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D9:G9)</f>
+        <v>6</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="26" t="s">
-        <v>279</v>
+        <v>314</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>280</v>
+        <v>315</v>
+      </c>
+      <c r="D10" s="23">
+        <v>1</v>
+      </c>
+      <c r="E10" s="23">
+        <v>0</v>
+      </c>
+      <c r="F10" s="23">
+        <v>1</v>
+      </c>
+      <c r="G10" s="23">
+        <v>2</v>
       </c>
       <c r="H10" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D10:G10)</f>
+        <v>4</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="26" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>315</v>
+        <v>327</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>339</v>
       </c>
       <c r="H11" s="24">
-        <f t="shared" si="0"/>
+        <f>SUM(D11:G11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="26" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>327</v>
+        <v>319</v>
+      </c>
+      <c r="D12" s="23">
+        <v>0</v>
+      </c>
+      <c r="E12" s="23">
+        <v>2</v>
+      </c>
+      <c r="F12" s="23">
+        <v>2</v>
+      </c>
+      <c r="G12" s="23">
+        <v>2</v>
       </c>
       <c r="H12" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D12:G12)</f>
+        <v>6</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="26" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>319</v>
+        <v>305</v>
+      </c>
+      <c r="D13" s="23">
+        <v>0</v>
+      </c>
+      <c r="E13" s="23">
+        <v>2</v>
+      </c>
+      <c r="F13" s="23">
+        <v>2</v>
+      </c>
+      <c r="G13" s="23">
+        <v>2</v>
       </c>
       <c r="H13" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D13:G13)</f>
+        <v>6</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="26" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>305</v>
+        <v>313</v>
+      </c>
+      <c r="D14" s="23">
+        <v>1</v>
+      </c>
+      <c r="E14" s="23">
+        <v>1</v>
+      </c>
+      <c r="F14" s="23">
+        <v>1</v>
+      </c>
+      <c r="G14" s="23">
+        <v>2</v>
       </c>
       <c r="H14" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D14:G14)</f>
+        <v>5</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="26" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>313</v>
+        <v>325</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1</v>
+      </c>
+      <c r="E15" s="23">
+        <v>1</v>
+      </c>
+      <c r="F15" s="23">
+        <v>1</v>
+      </c>
+      <c r="G15" s="23">
+        <v>1</v>
       </c>
       <c r="H15" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(D15:G15)</f>
+        <v>4</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="26" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>325</v>
+        <v>285</v>
+      </c>
+      <c r="D16" s="23">
+        <v>1</v>
+      </c>
+      <c r="E16" s="23">
+        <v>2</v>
+      </c>
+      <c r="F16" s="23">
+        <v>2</v>
+      </c>
+      <c r="G16" s="23">
+        <v>2</v>
       </c>
       <c r="H16" s="24">
-        <f t="shared" si="0"/>
+        <f>SUM(D16:G16)</f>
+        <v>7</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="26" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="D17" s="23">
+        <v>1</v>
+      </c>
+      <c r="E17" s="23">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="26" t="s">
-        <v>330</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>285</v>
+      <c r="F17" s="23">
+        <v>1</v>
+      </c>
+      <c r="G17" s="23">
+        <v>0</v>
       </c>
       <c r="H17" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D17:G17)</f>
+        <v>2</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="26" t="s">
-        <v>288</v>
+        <v>316</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>289</v>
+        <v>317</v>
+      </c>
+      <c r="D18" s="23">
+        <v>1</v>
+      </c>
+      <c r="E18" s="23">
+        <v>2</v>
+      </c>
+      <c r="F18" s="23">
+        <v>1</v>
+      </c>
+      <c r="G18" s="23">
+        <v>1</v>
       </c>
       <c r="H18" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D18:G18)</f>
+        <v>5</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="26" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>317</v>
+        <v>321</v>
+      </c>
+      <c r="D19" s="23">
+        <v>2</v>
+      </c>
+      <c r="E19" s="23">
+        <v>2</v>
+      </c>
+      <c r="F19" s="23">
+        <v>1</v>
+      </c>
+      <c r="G19" s="23">
+        <v>2</v>
       </c>
       <c r="H19" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D19:G19)</f>
+        <v>7</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="26" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>321</v>
+        <v>323</v>
+      </c>
+      <c r="D20" s="23">
+        <v>1</v>
+      </c>
+      <c r="E20" s="23">
+        <v>2</v>
+      </c>
+      <c r="F20" s="23">
+        <v>2</v>
+      </c>
+      <c r="G20" s="23">
+        <v>2</v>
       </c>
       <c r="H20" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D20:G20)</f>
+        <v>7</v>
+      </c>
+      <c r="I20" s="23" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="26" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>323</v>
+        <v>328</v>
+      </c>
+      <c r="D21" s="23">
+        <v>1</v>
+      </c>
+      <c r="E21" s="23">
+        <v>1</v>
+      </c>
+      <c r="F21" s="23">
+        <v>1</v>
+      </c>
+      <c r="G21" s="23">
+        <v>1</v>
       </c>
       <c r="H21" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D21:G21)</f>
+        <v>4</v>
+      </c>
+      <c r="I21" s="23" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="26" t="s">
         <v>283</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>284</v>
       </c>
+      <c r="D22" s="23">
+        <v>2</v>
+      </c>
+      <c r="E22" s="23">
+        <v>2</v>
+      </c>
+      <c r="F22" s="23">
+        <v>2</v>
+      </c>
+      <c r="G22" s="23">
+        <v>2</v>
+      </c>
       <c r="H22" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D22:G22)</f>
+        <v>8</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="26" t="s">
         <v>298</v>
       </c>
       <c r="B23" s="23" t="s">
         <v>299</v>
       </c>
+      <c r="D23" s="23">
+        <v>1</v>
+      </c>
+      <c r="E23" s="23">
+        <v>2</v>
+      </c>
+      <c r="F23" s="23">
+        <v>2</v>
+      </c>
+      <c r="G23" s="23">
+        <v>2</v>
+      </c>
       <c r="H23" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D23:G23)</f>
+        <v>7</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="26" t="s">
         <v>310</v>
       </c>
       <c r="B24" s="23" t="s">
         <v>311</v>
       </c>
+      <c r="D24" s="23">
+        <v>2</v>
+      </c>
+      <c r="E24" s="23">
+        <v>2</v>
+      </c>
+      <c r="F24" s="23">
+        <v>2</v>
+      </c>
+      <c r="G24" s="23">
+        <v>2</v>
+      </c>
       <c r="H24" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D24:G24)</f>
+        <v>8</v>
+      </c>
+      <c r="I24" s="23" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="26" t="s">
         <v>296</v>
       </c>
       <c r="B25" s="23" t="s">
         <v>297</v>
       </c>
+      <c r="D25" s="23">
+        <v>1</v>
+      </c>
+      <c r="E25" s="23">
+        <v>2</v>
+      </c>
+      <c r="F25" s="23">
+        <v>1</v>
+      </c>
+      <c r="G25" s="23">
+        <v>2</v>
+      </c>
       <c r="H25" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D25:G25)</f>
+        <v>6</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="26" t="s">
         <v>300</v>
       </c>
       <c r="B26" s="23" t="s">
         <v>301</v>
       </c>
+      <c r="D26" s="23">
+        <v>1</v>
+      </c>
+      <c r="E26" s="23">
+        <v>2</v>
+      </c>
+      <c r="F26" s="23">
+        <v>2</v>
+      </c>
+      <c r="G26" s="23">
+        <v>2</v>
+      </c>
       <c r="H26" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.15">
+        <f>SUM(D26:G26)</f>
+        <v>7</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="26" t="s">
         <v>286</v>
       </c>
       <c r="B27" s="23" t="s">
         <v>287</v>
       </c>
+      <c r="C27" s="23" t="s">
+        <v>355</v>
+      </c>
+      <c r="D27" s="23">
+        <v>0</v>
+      </c>
+      <c r="E27" s="23">
+        <v>0</v>
+      </c>
+      <c r="F27" s="23">
+        <v>0</v>
+      </c>
+      <c r="G27" s="23">
+        <v>0</v>
+      </c>
       <c r="H27" s="24">
-        <f t="shared" si="0"/>
+        <f>SUM(D27:G27)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A28" s="26"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A29" s="26"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A30" s="26"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A31" s="26"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A32" s="26"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.15">
@@ -6039,6 +6471,7 @@
     <dataValidation showInputMessage="1" showErrorMessage="1" promptTitle="Conceptual and Methodological Ri" prompt="How clearly and coherently is the contribution conceptually and methodologically grounded?_x000a_" sqref="G1" xr:uid="{00000000-0002-0000-0200-000004000000}"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>